<commit_message>
IPO Desk: M. K. Sons refreshed on FY26 results from the RHP - call Neutral -> Subscribe (close to the line)
FY26 (RHP via trackers): revenue Rs 538.73 cr, EBITDA Rs 82.93 cr, PAT Rs 51.79 cr,
net worth Rs 168.01 cr, borrowings Rs 68.44 cr, CFO Rs 15.40 cr, EPS Rs 12.13.
Fair value Rs 127 / 149 / 175 (was 103 / 120 / 141 on DRHP 9M annualised).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sh3XfYSpHMqTXgPXQV3Xds
</commit_message>
<xml_diff>
--- a/ipo-analysis/companies/m-k-sons-fine-jewels-ltd/M_K_SONS_FINE_JEWELS_LTD_01_Screening.xlsx
+++ b/ipo-analysis/companies/m-k-sons-fine-jewels-ltd/M_K_SONS_FINE_JEWELS_LTD_01_Screening.xlsx
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>46022</v>
+        <v>46112</v>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Price band, lot, issue split and dates from the NSE issue page; RHP not reachable, so DRHP (May-2026) figures are used</t>
+          <t>RHP not reachable; FY24-25 and Dec-25 detail from the DRHP (May-2026), FY26 headline figures from the RHP as reproduced by IPO trackers (29-Oct-2026)</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
@@ -1307,20 +1307,18 @@
         </is>
       </c>
       <c r="C5" s="16" t="n">
-        <v>24.912</v>
+        <v>217.323</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>217.323</v>
+        <v>351.28</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>351.28</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <v>360.821</v>
-      </c>
+        <v>538.73</v>
+      </c>
+      <c r="F5" s="16" t="n"/>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>p. 227</t>
+          <t>p. 227; FY26 from RHP as reproduced by IPO trackers (Finology, INDmoney, Paytm Money)</t>
         </is>
       </c>
     </row>
@@ -1331,17 +1329,13 @@
         </is>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.018</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="E6" s="16" t="n">
         <v>0.036</v>
       </c>
-      <c r="F6" s="16" t="n">
-        <v>0.024</v>
-      </c>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
       <c r="G6" s="7" t="inlineStr">
         <is>
           <t>p. 227</t>
@@ -1355,17 +1349,13 @@
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>1.725</v>
+        <v>10.832</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>10.832</v>
-      </c>
-      <c r="E7" s="16" t="n">
         <v>32.026</v>
       </c>
-      <c r="F7" s="16" t="n">
-        <v>39.946</v>
-      </c>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>p. 227</t>
@@ -1379,17 +1369,13 @@
         </is>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.483</v>
+        <v>2.789</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>2.789</v>
-      </c>
-      <c r="E8" s="16" t="n">
         <v>8.550000000000001</v>
       </c>
-      <c r="F8" s="16" t="n">
-        <v>11</v>
-      </c>
+      <c r="E8" s="16" t="n"/>
+      <c r="F8" s="16" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
           <t>p. 227</t>
@@ -1403,17 +1389,13 @@
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>-0.097</v>
+        <v>-0.122</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>-0.122</v>
-      </c>
-      <c r="E9" s="16" t="n">
         <v>0.213</v>
       </c>
-      <c r="F9" s="16" t="n">
-        <v>-0.219</v>
-      </c>
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="16" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>p. 227</t>
@@ -1427,20 +1409,18 @@
         </is>
       </c>
       <c r="C10" s="16" t="n">
-        <v>1.339</v>
+        <v>8.164999999999999</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>8.164999999999999</v>
+        <v>23.262</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>23.262</v>
-      </c>
-      <c r="F10" s="16" t="n">
-        <v>29.165</v>
-      </c>
+        <v>51.79</v>
+      </c>
+      <c r="F10" s="16" t="n"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>p. 227</t>
+          <t>p. 227; FY26 from RHP as reproduced by IPO trackers (Finology, INDmoney, Paytm Money)</t>
         </is>
       </c>
     </row>
@@ -1451,20 +1431,18 @@
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>-4.947</v>
+        <v>-23.557</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>-23.557</v>
+        <v>-9.531000000000001</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>-9.531000000000001</v>
-      </c>
-      <c r="F11" s="16" t="n">
-        <v>18.006</v>
-      </c>
+        <v>15.4</v>
+      </c>
+      <c r="F11" s="16" t="n"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>p. 228</t>
+          <t>p. 228; FY26 from RHP as reproduced by IPO trackers (Finology, INDmoney, Paytm Money)</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1458,8 @@
       <c r="D12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="16" t="n">
-        <v>0</v>
-      </c>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
           <t>p. 64</t>
@@ -1499,17 +1473,13 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>0.459</v>
+        <v>3.849</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>3.849</v>
-      </c>
-      <c r="E13" s="16" t="n">
         <v>21.715</v>
       </c>
-      <c r="F13" s="16" t="n">
-        <v>1.228</v>
-      </c>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>p. 64 (purchases from the promoter's proprietorship before its merger, a promoter-group hotel, and rent to the promoter)</t>
@@ -1523,20 +1493,18 @@
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>14.149</v>
+        <v>22.29</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>22.29</v>
+        <v>116.235</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>116.235</v>
-      </c>
-      <c r="F14" s="16" t="n">
-        <v>145.418</v>
-      </c>
+        <v>168.01</v>
+      </c>
+      <c r="F14" s="16" t="n"/>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>p. 226</t>
+          <t>p. 226; FY26 from RHP as reproduced by IPO trackers (Finology, INDmoney, Paytm Money)</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1515,13 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>0.13</v>
+        <v>0.589</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>0.589</v>
-      </c>
-      <c r="E15" s="16" t="n">
         <v>1.21</v>
       </c>
-      <c r="F15" s="16" t="n">
-        <v>3.422</v>
-      </c>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
       <c r="G15" s="7" t="inlineStr">
         <is>
           <t>p. 226</t>
@@ -1571,17 +1535,13 @@
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>44.812</v>
+        <v>87.48099999999999</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>87.48099999999999</v>
-      </c>
-      <c r="E16" s="16" t="n">
         <v>205.696</v>
       </c>
-      <c r="F16" s="16" t="n">
-        <v>240.592</v>
-      </c>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
           <t>p. 226</t>
@@ -1595,17 +1555,13 @@
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>21.644</v>
+        <v>26.055</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>26.055</v>
-      </c>
-      <c r="E17" s="16" t="n">
         <v>21.569</v>
       </c>
-      <c r="F17" s="16" t="n">
-        <v>28.609</v>
-      </c>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
       <c r="G17" s="7" t="inlineStr">
         <is>
           <t>p. 226</t>
@@ -1624,12 +1580,8 @@
       <c r="D18" s="16" t="n">
         <v>4.995</v>
       </c>
-      <c r="E18" s="16" t="n">
-        <v>4.995</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <v>4.995</v>
-      </c>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="n"/>
       <c r="G18" s="7" t="inlineStr">
         <is>
           <t>p. 63 (income-tax demands AY 2012-13 and 2017-18)</t>
@@ -1648,12 +1600,8 @@
       <c r="D19" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="16" t="n">
-        <v>0</v>
-      </c>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
       <c r="G19" s="7" t="inlineStr">
         <is>
           <t>p. 226</t>
@@ -2445,7 +2393,7 @@
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>Operating cash flow Rs -4.95 / -23.56 / -9.53 cr FY23-25 against PAT Rs 1.34 / 8.17 / 23.26 cr as inventory rose from Rs 44.81 cr to Rs 205.70 cr; 9M FY26 CFO +Rs 18.01 cr against PAT Rs 29.17 cr. Typical for a jewellery retailer stocking new showrooms; inventory days 122 -&gt; 178 -&gt; 205 (p. 101).</t>
+          <t>Operating cash flow Rs -23.56 / -9.53 cr FY24-25 (DRHP p. 228) and +Rs 15.40 cr in FY26 (RHP via trackers) against PAT Rs 8.17 / 23.26 / 51.79 cr; one tracker reports Q1 FY27 CFO about Rs -2.84 cr (single source). Typical for a jewellery retailer stocking new showrooms; most profit is reinvested in inventory.</t>
         </is>
       </c>
     </row>

</xml_diff>